<commit_message>
Final change in frontend
</commit_message>
<xml_diff>
--- a/frontend/public/Book4.xlsx
+++ b/frontend/public/Book4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdivy\Desktop\Webpage\New folder\frontend\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2254B049-E7D7-4121-B729-1019FE666321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D986B4B-7F62-4AC8-8006-2623E90B2294}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{4C397D62-E4CC-478D-8FFF-082C45C660ED}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
   <si>
     <t>s</t>
   </si>
@@ -118,37 +118,13 @@
   </si>
   <si>
     <t xml:space="preserve"> - </t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -225,12 +201,6 @@
     <font>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -475,19 +445,16 @@
     <xf numFmtId="1" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -496,11 +463,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -885,66 +855,64 @@
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="38" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="35" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="30" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="36" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="G1" s="36" t="s">
+      <c r="G1" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
       <c r="J1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="36" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="32" t="s">
+      <c r="B2" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="32" t="s">
+      <c r="C2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="D2" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="E2" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="34" t="s">
+      <c r="F2" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="32" t="s">
+      <c r="G2" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="34" t="s">
+      <c r="H2" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="34" t="s">
+      <c r="I2" s="32" t="s">
         <v>8</v>
       </c>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="31"/>
-      <c r="B3" s="32"/>
-      <c r="C3" s="33"/>
-      <c r="D3" s="35"/>
-      <c r="E3" s="35"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="35"/>
-      <c r="I3" s="35"/>
+      <c r="A3" s="37"/>
+      <c r="B3" s="33"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="34"/>
+      <c r="E3" s="34"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="33"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="34"/>
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.35">
@@ -957,12 +925,8 @@
       <c r="C4" s="5">
         <v>7.31</v>
       </c>
-      <c r="D4" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
       <c r="F4" s="5">
         <f>6.26* 1.025</f>
         <v>6.4164999999999992</v>
@@ -973,9 +937,7 @@
       <c r="H4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="I4" s="6"/>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.35">
@@ -988,24 +950,16 @@
       <c r="C5" s="5">
         <v>3.393424357142858</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
       <c r="F5" s="5">
         <v>5.0557547500000002</v>
       </c>
       <c r="G5" s="5">
         <v>3.4538353555645163</v>
       </c>
-      <c r="H5" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.35">
@@ -1018,24 +972,16 @@
       <c r="C6" s="5">
         <v>1.8359000000000003</v>
       </c>
-      <c r="D6" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
       <c r="F6" s="5">
         <v>1.6037571000000002</v>
       </c>
       <c r="G6" s="5">
         <v>1.7790445497</v>
       </c>
-      <c r="H6" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.35">
@@ -1048,24 +994,16 @@
       <c r="C7" s="5">
         <v>1.6107294000000001</v>
       </c>
-      <c r="D7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
       <c r="F7" s="5">
         <v>1.6783841999999998</v>
       </c>
       <c r="G7" s="5">
         <v>1.1114357646000002</v>
       </c>
-      <c r="H7" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
       <c r="J7" s="1"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.35">
@@ -1079,12 +1017,8 @@
         <f>23.8*1.025</f>
         <v>24.395</v>
       </c>
-      <c r="D8" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
       <c r="F8" s="7">
         <f>23.94*1.025</f>
         <v>24.538499999999999</v>
@@ -1093,12 +1027,8 @@
         <f>23.8*1.025</f>
         <v>24.395</v>
       </c>
-      <c r="H8" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
       <c r="J8" s="1"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.35">
@@ -1111,24 +1041,16 @@
       <c r="C9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
       <c r="F9" s="8" t="s">
         <v>17</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
       <c r="J9" s="1"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
@@ -1141,12 +1063,8 @@
       <c r="C10" s="10">
         <v>0.42</v>
       </c>
-      <c r="D10" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
       <c r="F10" s="10">
         <v>0.15</v>
       </c>
@@ -1154,12 +1072,8 @@
         <f>0.56+0.2</f>
         <v>0.76</v>
       </c>
-      <c r="H10" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
       <c r="J10" s="1"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
@@ -1172,12 +1086,8 @@
       <c r="C11" s="12">
         <v>0</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
       <c r="F11" s="12">
         <v>0</v>
       </c>
@@ -1185,12 +1095,8 @@
         <f>G7*([1]Sheet1!$D$5)+0.05</f>
         <v>6.6671536469000009E-2</v>
       </c>
-      <c r="H11" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.35">
@@ -1203,23 +1109,15 @@
       <c r="C12" s="13">
         <v>0</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
       <c r="F12" s="13"/>
       <c r="G12" s="13">
         <f>-([1]Sheet1!$D$18+[1]Sheet1!$D$19)*([1]Sheet1!$D$50+[1]Sheet1!$D$51)/1000000</f>
         <v>-1.698</v>
       </c>
-      <c r="H12" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
       <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
@@ -1233,12 +1131,8 @@
         <f>SUM(C4:C12)</f>
         <v>38.965053757142861</v>
       </c>
-      <c r="D13" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
       <c r="F13" s="15">
         <f>SUM(F4:F12)</f>
         <v>39.442896049999995</v>
@@ -1247,12 +1141,8 @@
         <f>SUM(G4:G12)</f>
         <v>39.170247482235297</v>
       </c>
-      <c r="H13" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -1265,26 +1155,18 @@
       <c r="C14" s="18">
         <v>1.36</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
       <c r="F14" s="18">
         <f>(((180*4542) + (650*2*180))/1000000)*1.05</f>
         <v>1.1041380000000001</v>
       </c>
-      <c r="G14" s="18" t="e">
+      <c r="G14" s="18">
         <f>((H14*I14)/1000000) - G13</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>29</v>
-      </c>
+        <v>-39.170247482235297</v>
+      </c>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
       <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
@@ -1297,22 +1179,14 @@
       <c r="C15" s="20">
         <v>0</v>
       </c>
-      <c r="D15" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
       <c r="F15" s="20"/>
       <c r="G15" s="20">
         <v>-0.8</v>
       </c>
-      <c r="H15" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
       <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
@@ -1326,19 +1200,15 @@
         <f>C13+C14+C15</f>
         <v>40.325053757142861</v>
       </c>
-      <c r="D16" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
       <c r="F16" s="22">
         <f>F13+F14+F15</f>
         <v>40.547034049999993</v>
       </c>
-      <c r="G16" s="22" t="e">
+      <c r="G16" s="22">
         <f>G13+G14+G15</f>
-        <v>#VALUE!</v>
+        <v>-0.8</v>
       </c>
       <c r="H16" s="23">
         <v>7250</v>
@@ -1359,19 +1229,15 @@
       <c r="C17" s="25">
         <v>0.68</v>
       </c>
-      <c r="D17" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
       <c r="F17" s="25">
         <f>((H17*I17)/1000000)-F16</f>
         <v>0.68502565836359253</v>
       </c>
-      <c r="G17" s="25" t="e">
+      <c r="G17" s="25">
         <f>(H17*I17)/1000000 - G16</f>
-        <v>#VALUE!</v>
+        <v>42.032059708363583</v>
       </c>
       <c r="H17" s="16">
         <f>H16+ (2 * [1]Sheet1!$D$46)</f>
@@ -1393,19 +1259,15 @@
       <c r="C18" s="25">
         <v>1.37</v>
       </c>
-      <c r="D18" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
       <c r="F18" s="25">
         <f>(H18*I18)/1000000-F16-F17</f>
         <v>1.3838230412827599</v>
       </c>
-      <c r="G18" s="25" t="e">
+      <c r="G18" s="25">
         <f>(H18*I18)/1000000 -G16-G17</f>
-        <v>#VALUE!</v>
+        <v>1.3838230412827599</v>
       </c>
       <c r="H18" s="16">
         <f>H17+[1]Sheet1!$D$47</f>
@@ -1428,26 +1290,20 @@
         <f>SUM(C16:C18)</f>
         <v>42.375053757142858</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>29</v>
-      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
       <c r="F19" s="28">
         <f>SUM(F16:F18)</f>
         <v>42.615882749646346</v>
       </c>
-      <c r="G19" s="28" t="e">
+      <c r="G19" s="28">
         <f>SUM(G16:G18)</f>
-        <v>#VALUE!</v>
+        <v>42.615882749646346</v>
       </c>
       <c r="H19" s="29" t="s">
         <v>28</v>
       </c>
-      <c r="I19" s="29" t="s">
-        <v>30</v>
-      </c>
+      <c r="I19" s="29"/>
       <c r="J19" s="1"/>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -1500,17 +1356,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:G3"/>
     <mergeCell ref="H2:H3"/>
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="G1:I1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>